<commit_message>
agrega funcionalidad de poder cambiar el nombre de columnas para que sea mas dinamico
</commit_message>
<xml_diff>
--- a/app/datos_pipeline/paso3_modelos.xlsx
+++ b/app/datos_pipeline/paso3_modelos.xlsx
@@ -455,19 +455,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11481.79</v>
+        <v>13400.4</v>
       </c>
       <c r="C2" t="n">
-        <v>35491.5</v>
+        <v>45378.01</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8452</v>
+        <v>0.7399</v>
       </c>
       <c r="E2" t="n">
-        <v>59.35</v>
+        <v>61.63</v>
       </c>
       <c r="F2" t="n">
-        <v>24.11</v>
+        <v>24.71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: reorganizar archivos en app/ y docs/, agregar app_settings
Mueve los archivos historicos a app/Archivos Historicos/, el manual de
usuario a docs/ y actualiza los datos del pipeline. Agrega
app/app_settings.json con las rutas de archivos configuradas.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/datos_pipeline/paso3_modelos.xlsx
+++ b/app/datos_pipeline/paso3_modelos.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,32 +429,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>modelo</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>SMAPE%</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Accuracy%</t>
         </is>
@@ -455,19 +467,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13400.4</v>
+        <v>30104.06</v>
       </c>
       <c r="C2" t="n">
-        <v>45378.01</v>
+        <v>73556.42</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7399</v>
+        <v>0.8265</v>
       </c>
       <c r="E2" t="n">
-        <v>61.63</v>
+        <v>44.34</v>
       </c>
       <c r="F2" t="n">
-        <v>24.71</v>
+        <v>31.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>